<commit_message>
Adding Updated Addressing plan now with DNS internal record names
</commit_message>
<xml_diff>
--- a/documents/Addressing_Plan/Cisco Team 3 Addressing Plan Updated.xlsx
+++ b/documents/Addressing_Plan/Cisco Team 3 Addressing Plan Updated.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10927"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bensmac/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rjpop\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{01DDE242-CA50-4A4B-AF74-2E7656FAF2C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CDA65316-268A-4105-958A-EC6576065770}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="600" windowWidth="28560" windowHeight="16340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1950" yWindow="1950" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="158">
   <si>
     <t>Cisco Team 3</t>
   </si>
@@ -492,6 +492,27 @@
   </si>
   <si>
     <t>Network Device Interface Addressing</t>
+  </si>
+  <si>
+    <t>Internal DNS Records</t>
+  </si>
+  <si>
+    <t>Hostname</t>
+  </si>
+  <si>
+    <t>IP</t>
+  </si>
+  <si>
+    <t>dhcp-dns.kfp.internal</t>
+  </si>
+  <si>
+    <t>radius.kfp.internal</t>
+  </si>
+  <si>
+    <t>ntp-syslog.kfp.internal</t>
+  </si>
+  <si>
+    <t>resource.kfp.internal</t>
   </si>
 </sst>
 </file>
@@ -709,6 +730,27 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -717,27 +759,6 @@
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1058,20 +1079,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I71"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21.5" customWidth="1"/>
-    <col min="2" max="2" width="28.33203125" customWidth="1"/>
-    <col min="3" max="3" width="20.1640625" customWidth="1"/>
-    <col min="4" max="4" width="17.83203125" customWidth="1"/>
-    <col min="5" max="5" width="30.5" customWidth="1"/>
+    <col min="1" max="1" width="21.42578125" customWidth="1"/>
+    <col min="2" max="2" width="28.28515625" customWidth="1"/>
+    <col min="3" max="3" width="20.140625" customWidth="1"/>
+    <col min="4" max="4" width="17.85546875" customWidth="1"/>
+    <col min="5" max="5" width="30.42578125" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
-    <col min="7" max="7" width="40.5" customWidth="1"/>
-    <col min="8" max="8" width="22.1640625" customWidth="1"/>
-    <col min="9" max="9" width="21.6640625" customWidth="1"/>
+    <col min="7" max="7" width="40.42578125" customWidth="1"/>
+    <col min="8" max="8" width="22.140625" customWidth="1"/>
+    <col min="9" max="9" width="21.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1079,7 +1100,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>2</v>
       </c>
@@ -1108,7 +1129,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>11</v>
       </c>
@@ -1137,7 +1158,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>20</v>
       </c>
@@ -1166,7 +1187,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>26</v>
       </c>
@@ -1195,7 +1216,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>33</v>
       </c>
@@ -1224,7 +1245,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>39</v>
       </c>
@@ -1253,7 +1274,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>45</v>
       </c>
@@ -1282,7 +1303,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
         <v>50</v>
       </c>
@@ -1311,7 +1332,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
         <v>58</v>
       </c>
@@ -1340,7 +1361,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
         <v>62</v>
       </c>
@@ -1369,7 +1390,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="10" t="s">
         <v>66</v>
       </c>
@@ -1398,7 +1419,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="5"/>
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
@@ -1407,116 +1428,149 @@
       <c r="G14" s="5"/>
       <c r="H14" s="5"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>71</v>
       </c>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
       <c r="D16" s="5"/>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F16" s="1" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>72</v>
       </c>
       <c r="B17" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="C17" s="20" t="s">
+      <c r="C17" s="29" t="s">
         <v>74</v>
       </c>
-      <c r="D17" s="20"/>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="D17" s="29"/>
+      <c r="F17" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="G17" s="24" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>75</v>
       </c>
       <c r="B18" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="C18" s="21" t="s">
+      <c r="C18" s="30" t="s">
         <v>77</v>
       </c>
-      <c r="D18" s="21"/>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="D18" s="30"/>
+      <c r="F18" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="G18" s="22" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>78</v>
       </c>
       <c r="B19" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="C19" s="21" t="s">
+      <c r="C19" s="30" t="s">
         <v>80</v>
       </c>
-      <c r="D19" s="21"/>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="D19" s="30"/>
+      <c r="F19" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="G19" s="22" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>81</v>
       </c>
       <c r="B20" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="C20" s="21" t="s">
+      <c r="C20" s="30" t="s">
         <v>83</v>
       </c>
-      <c r="D20" s="21"/>
-    </row>
-    <row r="21" spans="1:7" ht="52.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D20" s="30"/>
+      <c r="F20" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="G20" s="22" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>84</v>
       </c>
       <c r="B21" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="C21" s="22" t="s">
+      <c r="C21" s="31" t="s">
         <v>144</v>
       </c>
-      <c r="D21" s="22"/>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="D21" s="31"/>
+      <c r="F21" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="G21" s="22" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>86</v>
       </c>
       <c r="B22" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="C22" s="21" t="s">
+      <c r="C22" s="30" t="s">
         <v>88</v>
       </c>
-      <c r="D22" s="21"/>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="D22" s="30"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>89</v>
       </c>
       <c r="B23" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="C23" s="21" t="s">
+      <c r="C23" s="30" t="s">
         <v>91</v>
       </c>
-      <c r="D23" s="21"/>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="D23" s="30"/>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>92</v>
       </c>
       <c r="B24" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="C24" s="21" t="s">
+      <c r="C24" s="30" t="s">
         <v>94</v>
       </c>
-      <c r="D24" s="21"/>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="D24" s="30"/>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="8" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
         <v>96</v>
       </c>
@@ -1537,7 +1591,7 @@
       </c>
       <c r="G27" s="8"/>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>100</v>
       </c>
@@ -1557,7 +1611,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>103</v>
       </c>
@@ -1577,7 +1631,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="17" t="s">
         <v>106</v>
       </c>
@@ -1597,7 +1651,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="10" t="s">
         <v>109</v>
       </c>
@@ -1617,12 +1671,12 @@
         <v>36</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="8" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="9" t="s">
         <v>96</v>
       </c>
@@ -1636,7 +1690,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="10" t="s">
         <v>19</v>
       </c>
@@ -1654,7 +1708,7 @@
       </c>
       <c r="F35" s="1"/>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="10" t="s">
         <v>32</v>
       </c>
@@ -1668,7 +1722,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="10" t="s">
         <v>117</v>
       </c>
@@ -1682,7 +1736,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="10" t="s">
         <v>120</v>
       </c>
@@ -1696,7 +1750,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="10" t="s">
         <v>122</v>
       </c>
@@ -1710,7 +1764,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" s="10" t="s">
         <v>124</v>
       </c>
@@ -1724,24 +1778,24 @@
         <v>125</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A41" s="24" t="s">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A41" s="21" t="s">
         <v>126</v>
       </c>
-      <c r="B41" s="24" t="s">
+      <c r="B41" s="21" t="s">
         <v>142</v>
       </c>
-      <c r="C41" s="24" t="s">
+      <c r="C41" s="21" t="s">
         <v>127</v>
       </c>
-      <c r="D41" s="24" t="s">
+      <c r="D41" s="21" t="s">
         <v>128</v>
       </c>
       <c r="E41" s="25" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>139</v>
       </c>
@@ -1756,69 +1810,69 @@
       </c>
       <c r="E42" s="25"/>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A43" s="26" t="s">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A43" s="22" t="s">
         <v>139</v>
       </c>
-      <c r="B43" s="26" t="s">
+      <c r="B43" s="22" t="s">
         <v>145</v>
       </c>
-      <c r="C43" s="26" t="s">
+      <c r="C43" s="22" t="s">
         <v>146</v>
       </c>
-      <c r="D43" s="26" t="s">
+      <c r="D43" s="22" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="44" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="30" t="s">
+    <row r="44" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="28" t="s">
         <v>149</v>
       </c>
-      <c r="B44" s="30"/>
-      <c r="C44" s="30"/>
-      <c r="D44" s="30"/>
-      <c r="E44" s="30"/>
-      <c r="F44" s="31"/>
-      <c r="G44" s="31"/>
-      <c r="H44" s="31"/>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A45" s="30"/>
-      <c r="B45" s="30"/>
-      <c r="C45" s="30"/>
-      <c r="D45" s="30"/>
-      <c r="E45" s="30"/>
-      <c r="F45" s="31"/>
-      <c r="G45" s="31"/>
-      <c r="H45" s="31"/>
-    </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A46" s="30"/>
-      <c r="B46" s="30"/>
-      <c r="C46" s="30"/>
-      <c r="D46" s="30"/>
-      <c r="E46" s="30"/>
-      <c r="F46" s="31"/>
-      <c r="G46" s="31"/>
-      <c r="H46" s="31"/>
-    </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A47" s="31"/>
-      <c r="B47" s="31"/>
-      <c r="C47" s="31"/>
-      <c r="D47" s="31"/>
-      <c r="E47" s="31"/>
-      <c r="F47" s="31"/>
-      <c r="G47" s="31"/>
-      <c r="H47" s="31"/>
-    </row>
-    <row r="49" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B44" s="28"/>
+      <c r="C44" s="28"/>
+      <c r="D44" s="28"/>
+      <c r="E44" s="28"/>
+      <c r="F44" s="23"/>
+      <c r="G44" s="23"/>
+      <c r="H44" s="23"/>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A45" s="28"/>
+      <c r="B45" s="28"/>
+      <c r="C45" s="28"/>
+      <c r="D45" s="28"/>
+      <c r="E45" s="28"/>
+      <c r="F45" s="23"/>
+      <c r="G45" s="23"/>
+      <c r="H45" s="23"/>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A46" s="28"/>
+      <c r="B46" s="28"/>
+      <c r="C46" s="28"/>
+      <c r="D46" s="28"/>
+      <c r="E46" s="28"/>
+      <c r="F46" s="23"/>
+      <c r="G46" s="23"/>
+      <c r="H46" s="23"/>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A47" s="23"/>
+      <c r="B47" s="23"/>
+      <c r="C47" s="23"/>
+      <c r="D47" s="23"/>
+      <c r="E47" s="23"/>
+      <c r="F47" s="23"/>
+      <c r="G47" s="23"/>
+      <c r="H47" s="23"/>
+    </row>
+    <row r="49" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="8" t="s">
         <v>129</v>
       </c>
-      <c r="F49" s="23"/>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F49" s="20"/>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
         <v>98</v>
       </c>
@@ -1834,9 +1888,9 @@
       <c r="E50" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="F50" s="23"/>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F50" s="20"/>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="2">
         <v>10</v>
       </c>
@@ -1852,9 +1906,9 @@
       <c r="E51" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="F51" s="23"/>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F51" s="20"/>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="2">
         <v>20</v>
       </c>
@@ -1870,9 +1924,9 @@
       <c r="E52" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="F52" s="23"/>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F52" s="20"/>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="2">
         <v>30</v>
       </c>
@@ -1888,9 +1942,9 @@
       <c r="E53" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="F53" s="23"/>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F53" s="20"/>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="2">
         <v>50</v>
       </c>
@@ -1906,51 +1960,51 @@
       <c r="E54" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="F54" s="23"/>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A55" s="28" t="s">
+      <c r="F54" s="20"/>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" s="26" t="s">
         <v>138</v>
       </c>
-      <c r="B55" s="28"/>
-      <c r="C55" s="28"/>
-      <c r="D55" s="28"/>
-      <c r="E55" s="28"/>
-      <c r="F55" s="27"/>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A56" s="29"/>
-      <c r="B56" s="29"/>
-      <c r="C56" s="29"/>
-      <c r="D56" s="29"/>
-      <c r="E56" s="29"/>
-      <c r="F56" s="27"/>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A57" s="29"/>
-      <c r="B57" s="29"/>
-      <c r="C57" s="29"/>
-      <c r="D57" s="29"/>
-      <c r="E57" s="29"/>
-      <c r="F57" s="27"/>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A58" s="29"/>
-      <c r="B58" s="29"/>
-      <c r="C58" s="29"/>
-      <c r="D58" s="29"/>
-      <c r="E58" s="29"/>
-      <c r="F58" s="27"/>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A59" s="27"/>
-      <c r="B59" s="27"/>
-      <c r="C59" s="27"/>
-      <c r="D59" s="27"/>
-      <c r="E59" s="27"/>
-      <c r="F59" s="27"/>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B55" s="26"/>
+      <c r="C55" s="26"/>
+      <c r="D55" s="26"/>
+      <c r="E55" s="26"/>
+      <c r="F55" s="5"/>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" s="27"/>
+      <c r="B56" s="27"/>
+      <c r="C56" s="27"/>
+      <c r="D56" s="27"/>
+      <c r="E56" s="27"/>
+      <c r="F56" s="5"/>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" s="27"/>
+      <c r="B57" s="27"/>
+      <c r="C57" s="27"/>
+      <c r="D57" s="27"/>
+      <c r="E57" s="27"/>
+      <c r="F57" s="5"/>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" s="27"/>
+      <c r="B58" s="27"/>
+      <c r="C58" s="27"/>
+      <c r="D58" s="27"/>
+      <c r="E58" s="27"/>
+      <c r="F58" s="5"/>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" s="5"/>
+      <c r="B59" s="5"/>
+      <c r="C59" s="5"/>
+      <c r="D59" s="5"/>
+      <c r="E59" s="5"/>
+      <c r="F59" s="5"/>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" s="5"/>
       <c r="B60" s="5"/>
       <c r="C60" s="5"/>
@@ -1958,14 +2012,14 @@
       <c r="E60" s="5"/>
       <c r="F60" s="5"/>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B61" s="5"/>
       <c r="C61" s="5"/>
       <c r="D61" s="5"/>
       <c r="E61" s="5"/>
       <c r="F61" s="5"/>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" s="5"/>
       <c r="B62" s="5"/>
       <c r="C62" s="5"/>
@@ -1973,7 +2027,7 @@
       <c r="E62" s="5"/>
       <c r="F62" s="5"/>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" s="5"/>
       <c r="B63" s="5"/>
       <c r="C63" s="5"/>
@@ -1981,7 +2035,7 @@
       <c r="E63" s="5"/>
       <c r="F63" s="5"/>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" s="5"/>
       <c r="B64" s="5"/>
       <c r="C64" s="5"/>
@@ -1989,7 +2043,7 @@
       <c r="E64" s="5"/>
       <c r="F64" s="5"/>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="5"/>
       <c r="B65" s="5"/>
       <c r="C65" s="5"/>
@@ -1997,7 +2051,7 @@
       <c r="E65" s="5"/>
       <c r="F65" s="5"/>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="5"/>
       <c r="B66" s="5"/>
       <c r="C66" s="5"/>
@@ -2005,7 +2059,7 @@
       <c r="E66" s="5"/>
       <c r="F66" s="5"/>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="5"/>
       <c r="B67" s="5"/>
       <c r="C67" s="5"/>
@@ -2013,7 +2067,7 @@
       <c r="E67" s="5"/>
       <c r="F67" s="5"/>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" s="5"/>
       <c r="B68" s="5"/>
       <c r="C68" s="5"/>
@@ -2021,7 +2075,7 @@
       <c r="E68" s="5"/>
       <c r="F68" s="5"/>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" s="5"/>
       <c r="B69" s="5"/>
       <c r="C69" s="5"/>
@@ -2029,7 +2083,7 @@
       <c r="E69" s="5"/>
       <c r="F69" s="5"/>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" s="5"/>
       <c r="B70" s="5"/>
       <c r="C70" s="5"/>
@@ -2037,7 +2091,7 @@
       <c r="E70" s="5"/>
       <c r="F70" s="5"/>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" s="5"/>
       <c r="B71" s="5"/>
       <c r="C71" s="5"/>

</xml_diff>